<commit_message>
#28 eSpark And Client BOM updated.
</commit_message>
<xml_diff>
--- a/Design Files/Adv-OLED-v2.0/BOM/eSpark_BOM_OLED-v2.0.xlsx
+++ b/Design Files/Adv-OLED-v2.0/BOM/eSpark_BOM_OLED-v2.0.xlsx
@@ -5,7 +5,7 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\chrisbyrd-esp32iotproduct\Design Files\OLED-v2.0\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\chrisbyrd-esp32iotproduct\Design Files\Adv-OLED-v2.0\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="105">
   <si>
     <t>Component list</t>
   </si>
@@ -51,78 +51,36 @@
     <t>Capacitor</t>
   </si>
   <si>
-    <t>Diode</t>
-  </si>
-  <si>
     <t>Pogo Connector</t>
   </si>
   <si>
-    <t>Wire To Board Connector</t>
-  </si>
-  <si>
     <t>RGB LED</t>
   </si>
   <si>
-    <t>OLED</t>
-  </si>
-  <si>
     <t>Mosfet</t>
   </si>
   <si>
     <t>Resistor</t>
   </si>
   <si>
-    <t>Solder Bridge</t>
-  </si>
-  <si>
     <t>Designator</t>
   </si>
   <si>
-    <t>C1, C2, C3, C9</t>
-  </si>
-  <si>
     <t>C4, C5, C6, C7</t>
   </si>
   <si>
-    <t>C8</t>
-  </si>
-  <si>
-    <t>C11</t>
-  </si>
-  <si>
-    <t>D1</t>
-  </si>
-  <si>
     <t>J1</t>
   </si>
   <si>
-    <t>J2</t>
-  </si>
-  <si>
     <t>LED1</t>
   </si>
   <si>
-    <t>OLED1</t>
-  </si>
-  <si>
     <t>Q1</t>
   </si>
   <si>
-    <t>R1, R2, R3, R7</t>
-  </si>
-  <si>
     <t>R4</t>
   </si>
   <si>
-    <t>R5</t>
-  </si>
-  <si>
-    <t>R6</t>
-  </si>
-  <si>
-    <t>SB1</t>
-  </si>
-  <si>
     <t>SW1, SW2, SW3</t>
   </si>
   <si>
@@ -135,45 +93,15 @@
     <t>CAP CER 0.1UF 50V X5R 0402</t>
   </si>
   <si>
-    <t>CAP CER 4.7UF 10V X5R 0402</t>
-  </si>
-  <si>
-    <t>CAP CER 2.2UF 25V X5R 0402</t>
-  </si>
-  <si>
-    <t>80V Single 1.2V@100mA 4ns 100mA SOD-523 Switching Diode ROHS</t>
-  </si>
-  <si>
     <t>Pogo Pad 2.5mm 4 Pin</t>
   </si>
   <si>
-    <t>CONN HEADER SMD R/A 11POS 1.25MM</t>
-  </si>
-  <si>
     <t>SMD,3.5x3.5mm Light Emitting Diodes (LED) RoHS</t>
   </si>
   <si>
-    <t>SSD1306 0.96 - OLED Displays Modules ROHS</t>
-  </si>
-  <si>
     <t>50V 220mA 3.5Ω@10V,220mA 225mW 1.6V@1mA N Channel SOT-23 MOSFETs ROHS</t>
   </si>
   <si>
-    <t>RES SMD 10K OHM 0.1% 1/10W 0603</t>
-  </si>
-  <si>
-    <t>RES SMD 4.7K OHM 5% 1/10W 0402</t>
-  </si>
-  <si>
-    <t>RES 0 OHM JUMPER 1/16W 0402</t>
-  </si>
-  <si>
-    <t>±1% 412kΩ 0402 Chip Resistor - Surface Mount ROHS</t>
-  </si>
-  <si>
-    <t>Solder Bridge ON</t>
-  </si>
-  <si>
     <t>3mm 2mm Round Button 50mA Top3.65mm SPST 12V SMD Tactile Switches</t>
   </si>
   <si>
@@ -183,27 +111,15 @@
     <t>Cap-0402</t>
   </si>
   <si>
-    <t>SOD-523</t>
-  </si>
-  <si>
     <t>Pogo 4 Pin</t>
   </si>
   <si>
-    <t>53261-1171</t>
-  </si>
-  <si>
     <t>WS2812B-Mini</t>
   </si>
   <si>
-    <t>N096-2864KSWEG01-H30</t>
-  </si>
-  <si>
     <t>Sot-23</t>
   </si>
   <si>
-    <t>Res-0603</t>
-  </si>
-  <si>
     <t>Res-0402</t>
   </si>
   <si>
@@ -216,33 +132,12 @@
     <t>C1005X5R1H104K050BB</t>
   </si>
   <si>
-    <t>CC0402KRX5R6BB475</t>
-  </si>
-  <si>
-    <t>GRM155R61E225KE11D</t>
-  </si>
-  <si>
-    <t>1SS355WT</t>
-  </si>
-  <si>
     <t>POGO Connector 4 Pin</t>
   </si>
   <si>
     <t>BSS138</t>
   </si>
   <si>
-    <t>RT0603BRD0710KL</t>
-  </si>
-  <si>
-    <t>ERJ-2GEJ472X</t>
-  </si>
-  <si>
-    <t>RC0402FR-070RL</t>
-  </si>
-  <si>
-    <t>FRC0402F4123TS</t>
-  </si>
-  <si>
     <t>TS-1185EC-C-D-B</t>
   </si>
   <si>
@@ -255,30 +150,12 @@
     <t>TDK</t>
   </si>
   <si>
-    <t>Murata</t>
-  </si>
-  <si>
-    <t>CBI</t>
-  </si>
-  <si>
-    <t>Molex</t>
-  </si>
-  <si>
     <t>Worldsemi</t>
   </si>
   <si>
-    <t>Newvisio</t>
-  </si>
-  <si>
     <t>Slkor(SLKORMICRO Elec.)</t>
   </si>
   <si>
-    <t>Panasonic</t>
-  </si>
-  <si>
-    <t>FOJAN</t>
-  </si>
-  <si>
     <t>XKB</t>
   </si>
   <si>
@@ -291,33 +168,12 @@
     <t>C2181865</t>
   </si>
   <si>
-    <t>C326586</t>
-  </si>
-  <si>
-    <t>C385032</t>
-  </si>
-  <si>
-    <t>C585957</t>
-  </si>
-  <si>
     <t>C527089</t>
   </si>
   <si>
-    <t>C2890596</t>
-  </si>
-  <si>
     <t>C426569</t>
   </si>
   <si>
-    <t>C95204</t>
-  </si>
-  <si>
-    <t>C106231</t>
-  </si>
-  <si>
-    <t>C5126037</t>
-  </si>
-  <si>
     <t>C318893</t>
   </si>
   <si>
@@ -327,24 +183,9 @@
     <t>0.1uF</t>
   </si>
   <si>
-    <t>4.7uF</t>
-  </si>
-  <si>
-    <t>2.2uf</t>
-  </si>
-  <si>
     <t>10K</t>
   </si>
   <si>
-    <t>4.7K</t>
-  </si>
-  <si>
-    <t>0R</t>
-  </si>
-  <si>
-    <t>412K</t>
-  </si>
-  <si>
     <t>Quantity</t>
   </si>
   <si>
@@ -390,16 +231,109 @@
     <t>LCSC</t>
   </si>
   <si>
-    <t>C2836063</t>
-  </si>
-  <si>
     <t>Custom</t>
   </si>
   <si>
-    <t>0402WGF4701TCE</t>
-  </si>
-  <si>
-    <t>C25900</t>
+    <t>C9</t>
+  </si>
+  <si>
+    <t>R1, R2, R3</t>
+  </si>
+  <si>
+    <t>Q2</t>
+  </si>
+  <si>
+    <t>Trans Gp Bjt NPN 25V 1.5A 300MW 3-PIN SOT-23 T/r</t>
+  </si>
+  <si>
+    <t>SOT-23</t>
+  </si>
+  <si>
+    <t>SS8050-G</t>
+  </si>
+  <si>
+    <t>Comchip</t>
+  </si>
+  <si>
+    <t>C105433</t>
+  </si>
+  <si>
+    <t>RES 1K OHM 1% 1/20W 0201</t>
+  </si>
+  <si>
+    <t>Res-0201</t>
+  </si>
+  <si>
+    <t>RC0201FR-071KP</t>
+  </si>
+  <si>
+    <t>1K</t>
+  </si>
+  <si>
+    <t>R5, R6, R7, R8</t>
+  </si>
+  <si>
+    <t>RES SMD 10 OHM 1% 1/5W 0402</t>
+  </si>
+  <si>
+    <t>CRCW040210R0FKEDHP</t>
+  </si>
+  <si>
+    <t>Vishay Dale</t>
+  </si>
+  <si>
+    <t>C4013850</t>
+  </si>
+  <si>
+    <t>10R</t>
+  </si>
+  <si>
+    <t>FPC Connector</t>
+  </si>
+  <si>
+    <t>J2, J3</t>
+  </si>
+  <si>
+    <t>Clamshell -25℃~+85℃ 18P Bottom Contact Surface Mount 0.5mm SMD,P=0.5mm FFC/FPC Connectors ROHS</t>
+  </si>
+  <si>
+    <t>F0502-B-18-15T-R</t>
+  </si>
+  <si>
+    <t>XFCN</t>
+  </si>
+  <si>
+    <t>C2889974</t>
+  </si>
+  <si>
+    <t>RC0201FR-0710KL</t>
+  </si>
+  <si>
+    <t>RES SMD 10K OHM 1% 1/20W 0201</t>
+  </si>
+  <si>
+    <t>C106225</t>
+  </si>
+  <si>
+    <t>C138165</t>
+  </si>
+  <si>
+    <t>RC0201FR-071KL</t>
+  </si>
+  <si>
+    <t>Peripheral</t>
+  </si>
+  <si>
+    <t>0.3mm~0.3mm 18 0.5mm Same Side 5cm P=0.5mm FFC/FPC Connect Cables ROHS</t>
+  </si>
+  <si>
+    <t>JS05A-18P-050-4-8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JUSHUO </t>
+  </si>
+  <si>
+    <t>C2857498</t>
   </si>
 </sst>
 </file>
@@ -871,7 +805,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="76">
+  <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1032,6 +966,21 @@
     <xf numFmtId="0" fontId="18" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="17" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1063,24 +1012,6 @@
     <xf numFmtId="0" fontId="20" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="22" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1424,7 +1355,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:S27"/>
+  <dimension ref="A1:S23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="26" customWidth="1"/>
@@ -1445,6 +1376,7 @@
     <col min="17" max="17" width="19.28515625" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="16.5703125" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="26.85546875" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="25.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1458,15 +1390,15 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
-      <c r="K1" s="60"/>
-      <c r="L1" s="60"/>
-      <c r="M1" s="60"/>
-      <c r="N1" s="60"/>
-      <c r="O1" s="60"/>
-      <c r="P1" s="60"/>
-      <c r="Q1" s="60"/>
-      <c r="R1" s="60"/>
-      <c r="S1" s="61"/>
+      <c r="K1" s="65"/>
+      <c r="L1" s="65"/>
+      <c r="M1" s="65"/>
+      <c r="N1" s="65"/>
+      <c r="O1" s="65"/>
+      <c r="P1" s="65"/>
+      <c r="Q1" s="65"/>
+      <c r="R1" s="65"/>
+      <c r="S1" s="66"/>
     </row>
     <row r="2" spans="1:19" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -1477,7 +1409,7 @@
       </c>
       <c r="E2" s="11"/>
       <c r="F2" s="55" t="s">
-        <v>120</v>
+        <v>67</v>
       </c>
       <c r="G2" s="12"/>
       <c r="H2" s="4"/>
@@ -1502,7 +1434,7 @@
       </c>
       <c r="E3" s="13"/>
       <c r="F3" s="56" t="s">
-        <v>121</v>
+        <v>68</v>
       </c>
       <c r="G3" s="13"/>
       <c r="H3" s="5"/>
@@ -1516,7 +1448,7 @@
       <c r="P3" s="5"/>
       <c r="Q3" s="5"/>
       <c r="R3" s="5"/>
-      <c r="S3" s="62"/>
+      <c r="S3" s="67"/>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -1527,7 +1459,7 @@
       </c>
       <c r="E4" s="13"/>
       <c r="F4" s="57" t="s">
-        <v>121</v>
+        <v>68</v>
       </c>
       <c r="G4" s="14"/>
       <c r="H4" s="7"/>
@@ -1541,7 +1473,7 @@
       <c r="P4" s="6"/>
       <c r="Q4" s="6"/>
       <c r="R4" s="6"/>
-      <c r="S4" s="63"/>
+      <c r="S4" s="68"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -1566,7 +1498,7 @@
       <c r="P5" s="6"/>
       <c r="Q5" s="6"/>
       <c r="R5" s="6"/>
-      <c r="S5" s="63"/>
+      <c r="S5" s="68"/>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -1587,7 +1519,7 @@
       <c r="P6" s="6"/>
       <c r="Q6" s="6"/>
       <c r="R6" s="6"/>
-      <c r="S6" s="63"/>
+      <c r="S6" s="68"/>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -1608,7 +1540,7 @@
       <c r="P7" s="8"/>
       <c r="Q7" s="8"/>
       <c r="R7" s="8"/>
-      <c r="S7" s="63"/>
+      <c r="S7" s="68"/>
     </row>
     <row r="8" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -1629,7 +1561,7 @@
       <c r="P8" s="8"/>
       <c r="Q8" s="8"/>
       <c r="R8" s="8"/>
-      <c r="S8" s="63"/>
+      <c r="S8" s="68"/>
     </row>
     <row r="9" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -1640,423 +1572,425 @@
         <v>8</v>
       </c>
       <c r="D9" s="30" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="E9" s="30" t="s">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="F9" s="30" t="s">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="G9" s="30" t="s">
+        <v>34</v>
+      </c>
+      <c r="H9" s="30" t="s">
+        <v>40</v>
+      </c>
+      <c r="I9" s="30" t="s">
+        <v>56</v>
+      </c>
+      <c r="J9" s="30" t="s">
+        <v>46</v>
+      </c>
+      <c r="K9" s="60" t="s">
+        <v>57</v>
+      </c>
+      <c r="L9" s="30" t="s">
+        <v>55</v>
+      </c>
+      <c r="M9" s="30" t="s">
+        <v>58</v>
+      </c>
+      <c r="N9" s="30" t="s">
+        <v>59</v>
+      </c>
+      <c r="O9" s="30" t="s">
+        <v>60</v>
+      </c>
+      <c r="P9" s="30" t="s">
+        <v>61</v>
+      </c>
+      <c r="Q9" s="30" t="s">
         <v>62</v>
       </c>
-      <c r="H9" s="30" t="s">
-        <v>75</v>
-      </c>
-      <c r="I9" s="30" t="s">
-        <v>109</v>
-      </c>
-      <c r="J9" s="30" t="s">
-        <v>87</v>
-      </c>
-      <c r="K9" s="70" t="s">
-        <v>110</v>
-      </c>
-      <c r="L9" s="30" t="s">
-        <v>108</v>
-      </c>
-      <c r="M9" s="30" t="s">
-        <v>111</v>
-      </c>
-      <c r="N9" s="30" t="s">
-        <v>112</v>
-      </c>
-      <c r="O9" s="30" t="s">
-        <v>113</v>
-      </c>
-      <c r="P9" s="30" t="s">
-        <v>114</v>
-      </c>
-      <c r="Q9" s="30" t="s">
-        <v>115</v>
-      </c>
       <c r="R9" s="30" t="s">
-        <v>116</v>
+        <v>63</v>
       </c>
       <c r="S9" s="30" t="s">
-        <v>117</v>
+        <v>64</v>
       </c>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A10" s="1"/>
-      <c r="B10" s="46">
-        <f>ROW(B10) - ROW($B$9)</f>
+      <c r="B10" s="47">
+        <f t="shared" ref="B10:B20" si="0">ROW(B10) - ROW($B$9)</f>
         <v>1</v>
       </c>
       <c r="C10" s="54" t="s">
         <v>9</v>
       </c>
-      <c r="D10" s="37" t="s">
-        <v>19</v>
-      </c>
-      <c r="E10" s="37" t="s">
+      <c r="D10" s="51" t="s">
+        <v>15</v>
+      </c>
+      <c r="E10" s="51" t="s">
+        <v>23</v>
+      </c>
+      <c r="F10" s="51" t="s">
+        <v>29</v>
+      </c>
+      <c r="G10" s="51" t="s">
         <v>36</v>
       </c>
-      <c r="F10" s="37" t="s">
+      <c r="H10" s="51" t="s">
+        <v>42</v>
+      </c>
+      <c r="I10" s="51" t="s">
+        <v>66</v>
+      </c>
+      <c r="J10" s="51" t="s">
+        <v>48</v>
+      </c>
+      <c r="K10" s="51" t="s">
         <v>53</v>
       </c>
-      <c r="G10" s="37" t="s">
-        <v>63</v>
-      </c>
-      <c r="H10" s="37" t="s">
-        <v>76</v>
-      </c>
-      <c r="I10" s="37" t="s">
-        <v>119</v>
-      </c>
-      <c r="J10" s="37" t="s">
-        <v>88</v>
-      </c>
-      <c r="K10" s="37" t="s">
-        <v>100</v>
-      </c>
-      <c r="L10" s="37">
+      <c r="L10" s="51">
         <v>4</v>
       </c>
-      <c r="M10" s="37">
-        <f>L10*5</f>
+      <c r="M10" s="51">
+        <f t="shared" ref="M10" si="1">L10*5</f>
         <v>20</v>
       </c>
-      <c r="N10" s="37">
-        <v>100</v>
-      </c>
-      <c r="O10" s="73" t="s">
-        <v>122</v>
-      </c>
-      <c r="P10" s="38">
-        <v>2.3999999999999998E-3</v>
-      </c>
-      <c r="Q10" s="38">
-        <f>P10*N10</f>
-        <v>0.24</v>
-      </c>
-      <c r="R10" s="37"/>
-      <c r="S10" s="50"/>
+      <c r="N10" s="51">
+        <v>25</v>
+      </c>
+      <c r="O10" s="62" t="s">
+        <v>69</v>
+      </c>
+      <c r="P10" s="52">
+        <v>9.5699999999999993E-2</v>
+      </c>
+      <c r="Q10" s="52">
+        <f t="shared" ref="Q10" si="2">P10*N10</f>
+        <v>2.3924999999999996</v>
+      </c>
+      <c r="R10" s="51"/>
+      <c r="S10" s="51"/>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A11" s="1"/>
-      <c r="B11" s="47">
-        <f t="shared" ref="B11:B25" si="0">ROW(B11) - ROW($B$9)</f>
+      <c r="B11" s="46">
+        <f>ROW(B11) - ROW($B$9)</f>
         <v>2</v>
       </c>
       <c r="C11" s="54" t="s">
         <v>9</v>
       </c>
-      <c r="D11" s="51" t="s">
-        <v>20</v>
-      </c>
-      <c r="E11" s="51" t="s">
-        <v>37</v>
-      </c>
-      <c r="F11" s="51" t="s">
-        <v>53</v>
-      </c>
-      <c r="G11" s="51" t="s">
-        <v>64</v>
-      </c>
-      <c r="H11" s="51" t="s">
-        <v>77</v>
-      </c>
-      <c r="I11" s="51" t="s">
-        <v>119</v>
-      </c>
-      <c r="J11" s="51" t="s">
-        <v>89</v>
-      </c>
-      <c r="K11" s="51" t="s">
-        <v>101</v>
-      </c>
-      <c r="L11" s="51">
-        <v>4</v>
-      </c>
-      <c r="M11" s="51">
-        <f t="shared" ref="M11" si="1">L11*5</f>
-        <v>20</v>
-      </c>
-      <c r="N11" s="51">
-        <v>25</v>
-      </c>
-      <c r="O11" s="73" t="s">
-        <v>122</v>
-      </c>
-      <c r="P11" s="52">
-        <v>9.5699999999999993E-2</v>
-      </c>
-      <c r="Q11" s="52">
-        <f t="shared" ref="Q11" si="2">P11*N11</f>
-        <v>2.3924999999999996</v>
-      </c>
-      <c r="R11" s="51"/>
-      <c r="S11" s="51"/>
+      <c r="D11" s="37" t="s">
+        <v>71</v>
+      </c>
+      <c r="E11" s="37" t="s">
+        <v>22</v>
+      </c>
+      <c r="F11" s="37" t="s">
+        <v>29</v>
+      </c>
+      <c r="G11" s="37" t="s">
+        <v>35</v>
+      </c>
+      <c r="H11" s="37" t="s">
+        <v>41</v>
+      </c>
+      <c r="I11" s="37" t="s">
+        <v>66</v>
+      </c>
+      <c r="J11" s="37" t="s">
+        <v>47</v>
+      </c>
+      <c r="K11" s="37" t="s">
+        <v>52</v>
+      </c>
+      <c r="L11" s="37">
+        <v>1</v>
+      </c>
+      <c r="M11" s="37">
+        <f>L11*5</f>
+        <v>5</v>
+      </c>
+      <c r="N11" s="37">
+        <v>100</v>
+      </c>
+      <c r="O11" s="62" t="s">
+        <v>69</v>
+      </c>
+      <c r="P11" s="38">
+        <v>2.3999999999999998E-3</v>
+      </c>
+      <c r="Q11" s="38">
+        <f>P11*N11</f>
+        <v>0.24</v>
+      </c>
+      <c r="R11" s="37"/>
+      <c r="S11" s="50"/>
     </row>
     <row r="12" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A12" s="1"/>
-      <c r="B12" s="46">
-        <f>ROW(B12) - ROW($B$9)</f>
+      <c r="B12" s="47">
+        <f t="shared" si="0"/>
         <v>3</v>
       </c>
       <c r="C12" s="54" t="s">
-        <v>9</v>
-      </c>
-      <c r="D12" s="37" t="s">
-        <v>21</v>
-      </c>
-      <c r="E12" s="37" t="s">
-        <v>38</v>
-      </c>
-      <c r="F12" s="37" t="s">
-        <v>53</v>
-      </c>
-      <c r="G12" s="37" t="s">
-        <v>65</v>
-      </c>
-      <c r="H12" s="37" t="s">
-        <v>76</v>
-      </c>
-      <c r="I12" s="37" t="s">
-        <v>119</v>
-      </c>
-      <c r="J12" s="37" t="s">
-        <v>90</v>
-      </c>
-      <c r="K12" s="37" t="s">
-        <v>102</v>
-      </c>
-      <c r="L12" s="37">
+        <v>10</v>
+      </c>
+      <c r="D12" s="61" t="s">
+        <v>16</v>
+      </c>
+      <c r="E12" s="61" t="s">
+        <v>24</v>
+      </c>
+      <c r="F12" s="61" t="s">
+        <v>30</v>
+      </c>
+      <c r="G12" s="61" t="s">
+        <v>37</v>
+      </c>
+      <c r="H12" s="61" t="s">
+        <v>66</v>
+      </c>
+      <c r="I12" s="61" t="s">
+        <v>66</v>
+      </c>
+      <c r="J12" s="61" t="s">
+        <v>66</v>
+      </c>
+      <c r="K12" s="61" t="s">
+        <v>66</v>
+      </c>
+      <c r="L12" s="61">
         <v>1</v>
       </c>
-      <c r="M12" s="37">
-        <f>L12*5</f>
+      <c r="M12" s="61">
+        <f t="shared" ref="M12:M13" si="3">L12*5</f>
         <v>5</v>
       </c>
-      <c r="N12" s="37">
-        <v>50</v>
-      </c>
-      <c r="O12" s="73" t="s">
-        <v>122</v>
-      </c>
-      <c r="P12" s="38">
-        <v>1.46E-2</v>
-      </c>
-      <c r="Q12" s="38">
-        <f>P12*N12</f>
-        <v>0.73</v>
-      </c>
-      <c r="R12" s="37"/>
-      <c r="S12" s="59"/>
+      <c r="N12" s="61" t="s">
+        <v>66</v>
+      </c>
+      <c r="O12" s="61" t="s">
+        <v>66</v>
+      </c>
+      <c r="P12" s="61" t="s">
+        <v>66</v>
+      </c>
+      <c r="Q12" s="61" t="s">
+        <v>66</v>
+      </c>
+      <c r="R12" s="61" t="s">
+        <v>66</v>
+      </c>
+      <c r="S12" s="61" t="s">
+        <v>66</v>
+      </c>
     </row>
-    <row r="13" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:19" ht="48" x14ac:dyDescent="0.25">
       <c r="A13" s="1"/>
       <c r="B13" s="47">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="C13" s="54" t="s">
-        <v>9</v>
+        <v>89</v>
       </c>
       <c r="D13" s="51" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E13" s="51" t="s">
-        <v>39</v>
+        <v>91</v>
       </c>
       <c r="F13" s="51" t="s">
-        <v>53</v>
+        <v>70</v>
       </c>
       <c r="G13" s="51" t="s">
-        <v>66</v>
+        <v>92</v>
       </c>
       <c r="H13" s="51" t="s">
-        <v>78</v>
+        <v>93</v>
       </c>
       <c r="I13" s="51" t="s">
-        <v>119</v>
+        <v>66</v>
       </c>
       <c r="J13" s="51" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="K13" s="51" t="s">
-        <v>103</v>
+        <v>66</v>
       </c>
       <c r="L13" s="51">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M13" s="51">
-        <f t="shared" ref="M13" si="3">L13*5</f>
-        <v>5</v>
+        <f t="shared" si="3"/>
+        <v>10</v>
       </c>
       <c r="N13" s="51">
-        <v>20</v>
-      </c>
-      <c r="O13" s="73" t="s">
-        <v>122</v>
+        <v>15</v>
+      </c>
+      <c r="O13" s="63" t="s">
+        <v>69</v>
       </c>
       <c r="P13" s="52">
-        <v>3.1699999999999999E-2</v>
+        <v>9.7500000000000003E-2</v>
       </c>
       <c r="Q13" s="52">
         <f t="shared" ref="Q13" si="4">P13*N13</f>
-        <v>0.63400000000000001</v>
+        <v>1.4625000000000001</v>
       </c>
       <c r="R13" s="51"/>
       <c r="S13" s="59"/>
     </row>
     <row r="14" spans="1:19" ht="24" x14ac:dyDescent="0.25">
       <c r="A14" s="1"/>
-      <c r="B14" s="46">
-        <f>ROW(B14) - ROW($B$9)</f>
+      <c r="B14" s="47">
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="C14" s="53" t="s">
+      <c r="C14" s="54" t="s">
+        <v>11</v>
+      </c>
+      <c r="D14" s="51" t="s">
+        <v>17</v>
+      </c>
+      <c r="E14" s="51" t="s">
+        <v>25</v>
+      </c>
+      <c r="F14" s="51" t="s">
+        <v>70</v>
+      </c>
+      <c r="G14" s="51" t="s">
+        <v>31</v>
+      </c>
+      <c r="H14" s="51" t="s">
+        <v>43</v>
+      </c>
+      <c r="I14" s="51" t="s">
+        <v>66</v>
+      </c>
+      <c r="J14" s="51" t="s">
+        <v>49</v>
+      </c>
+      <c r="K14" s="51" t="s">
+        <v>66</v>
+      </c>
+      <c r="L14" s="51">
+        <v>1</v>
+      </c>
+      <c r="M14" s="51">
+        <f t="shared" ref="M14" si="5">L14*5</f>
+        <v>5</v>
+      </c>
+      <c r="N14" s="51">
         <v>10</v>
       </c>
-      <c r="D14" s="37" t="s">
-        <v>23</v>
-      </c>
-      <c r="E14" s="37" t="s">
-        <v>40</v>
-      </c>
-      <c r="F14" s="37" t="s">
-        <v>54</v>
-      </c>
-      <c r="G14" s="37" t="s">
-        <v>67</v>
-      </c>
-      <c r="H14" s="37" t="s">
-        <v>79</v>
-      </c>
-      <c r="I14" s="37"/>
-      <c r="J14" s="37" t="s">
-        <v>123</v>
-      </c>
-      <c r="K14" s="37" t="s">
-        <v>119</v>
-      </c>
-      <c r="L14" s="37">
-        <v>1</v>
-      </c>
-      <c r="M14" s="37">
-        <f>L14*5</f>
-        <v>5</v>
-      </c>
-      <c r="N14" s="37">
-        <v>50</v>
-      </c>
-      <c r="O14" s="73" t="s">
-        <v>122</v>
-      </c>
-      <c r="P14" s="38">
-        <v>9.9000000000000008E-3</v>
-      </c>
-      <c r="Q14" s="38">
-        <f>P14*N14</f>
-        <v>0.49500000000000005</v>
-      </c>
-      <c r="R14" s="37"/>
+      <c r="O14" s="62" t="s">
+        <v>69</v>
+      </c>
+      <c r="P14" s="52">
+        <v>0.1176</v>
+      </c>
+      <c r="Q14" s="52">
+        <f t="shared" ref="Q14" si="6">P14*N14</f>
+        <v>1.1759999999999999</v>
+      </c>
+      <c r="R14" s="51"/>
       <c r="S14" s="59"/>
     </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:19" ht="36" x14ac:dyDescent="0.25">
       <c r="A15" s="1"/>
       <c r="B15" s="47">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
       <c r="C15" s="54" t="s">
-        <v>11</v>
-      </c>
-      <c r="D15" s="71" t="s">
-        <v>24</v>
-      </c>
-      <c r="E15" s="71" t="s">
-        <v>41</v>
-      </c>
-      <c r="F15" s="71" t="s">
-        <v>55</v>
-      </c>
-      <c r="G15" s="71" t="s">
-        <v>68</v>
-      </c>
-      <c r="H15" s="71" t="s">
-        <v>119</v>
-      </c>
-      <c r="I15" s="71" t="s">
-        <v>119</v>
-      </c>
-      <c r="J15" s="71" t="s">
-        <v>119</v>
-      </c>
-      <c r="K15" s="71" t="s">
-        <v>119</v>
-      </c>
-      <c r="L15" s="71">
+        <v>12</v>
+      </c>
+      <c r="D15" s="51" t="s">
+        <v>18</v>
+      </c>
+      <c r="E15" s="51" t="s">
+        <v>26</v>
+      </c>
+      <c r="F15" s="51" t="s">
+        <v>32</v>
+      </c>
+      <c r="G15" s="51" t="s">
+        <v>38</v>
+      </c>
+      <c r="H15" s="51" t="s">
+        <v>44</v>
+      </c>
+      <c r="I15" s="51" t="s">
+        <v>66</v>
+      </c>
+      <c r="J15" s="51" t="s">
+        <v>50</v>
+      </c>
+      <c r="K15" s="51" t="s">
+        <v>66</v>
+      </c>
+      <c r="L15" s="51">
         <v>1</v>
       </c>
-      <c r="M15" s="71">
-        <f t="shared" ref="M15" si="5">L15*5</f>
+      <c r="M15" s="51">
+        <f t="shared" ref="M15" si="7">L15*5</f>
         <v>5</v>
       </c>
-      <c r="N15" s="71" t="s">
-        <v>119</v>
-      </c>
-      <c r="O15" s="71" t="s">
-        <v>119</v>
-      </c>
-      <c r="P15" s="71" t="s">
-        <v>119</v>
-      </c>
-      <c r="Q15" s="71" t="s">
-        <v>119</v>
-      </c>
-      <c r="R15" s="71" t="s">
-        <v>119</v>
-      </c>
-      <c r="S15" s="71" t="s">
-        <v>119</v>
-      </c>
+      <c r="N15" s="51">
+        <v>20</v>
+      </c>
+      <c r="O15" s="62" t="s">
+        <v>69</v>
+      </c>
+      <c r="P15" s="52">
+        <v>2.1499999999999998E-2</v>
+      </c>
+      <c r="Q15" s="52">
+        <f t="shared" ref="Q15" si="8">P15*N15</f>
+        <v>0.42999999999999994</v>
+      </c>
+      <c r="R15" s="51"/>
+      <c r="S15" s="59"/>
     </row>
-    <row r="16" spans="1:19" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:19" ht="24" x14ac:dyDescent="0.25">
       <c r="A16" s="1"/>
       <c r="B16" s="46">
         <f>ROW(B16) - ROW($B$9)</f>
         <v>7</v>
       </c>
-      <c r="C16" s="53" t="s">
+      <c r="C16" s="54" t="s">
         <v>12</v>
       </c>
       <c r="D16" s="37" t="s">
-        <v>25</v>
+        <v>73</v>
       </c>
       <c r="E16" s="37" t="s">
-        <v>42</v>
+        <v>74</v>
       </c>
       <c r="F16" s="37" t="s">
-        <v>124</v>
+        <v>75</v>
       </c>
       <c r="G16" s="37" t="s">
-        <v>56</v>
+        <v>76</v>
       </c>
       <c r="H16" s="37" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="I16" s="37" t="s">
-        <v>119</v>
+        <v>66</v>
       </c>
       <c r="J16" s="37" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
       <c r="K16" s="37" t="s">
-        <v>119</v>
+        <v>66</v>
       </c>
       <c r="L16" s="37">
         <v>1</v>
@@ -2066,106 +2000,110 @@
         <v>5</v>
       </c>
       <c r="N16" s="37">
-        <v>6</v>
-      </c>
-      <c r="O16" s="73" t="s">
-        <v>122</v>
+        <v>50</v>
+      </c>
+      <c r="O16" s="62" t="s">
+        <v>69</v>
       </c>
       <c r="P16" s="38">
-        <v>0.36749999999999999</v>
+        <v>1.54E-2</v>
       </c>
       <c r="Q16" s="38">
         <f>P16*N16</f>
-        <v>2.2050000000000001</v>
+        <v>0.77</v>
       </c>
       <c r="R16" s="37"/>
       <c r="S16" s="59"/>
     </row>
-    <row r="17" spans="1:19" ht="24" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A17" s="1"/>
       <c r="B17" s="47">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="B17" si="9">ROW(B17) - ROW($B$9)</f>
         <v>8</v>
       </c>
       <c r="C17" s="54" t="s">
         <v>13</v>
       </c>
       <c r="D17" s="51" t="s">
-        <v>26</v>
+        <v>72</v>
       </c>
       <c r="E17" s="51" t="s">
-        <v>43</v>
+        <v>96</v>
       </c>
       <c r="F17" s="51" t="s">
-        <v>124</v>
+        <v>80</v>
       </c>
       <c r="G17" s="51" t="s">
-        <v>57</v>
+        <v>95</v>
       </c>
       <c r="H17" s="51" t="s">
-        <v>81</v>
+        <v>41</v>
       </c>
       <c r="I17" s="51" t="s">
-        <v>119</v>
+        <v>66</v>
       </c>
       <c r="J17" s="51" t="s">
-        <v>93</v>
-      </c>
-      <c r="K17" s="51"/>
+        <v>97</v>
+      </c>
+      <c r="K17" s="51" t="s">
+        <v>54</v>
+      </c>
       <c r="L17" s="51">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M17" s="51">
-        <f t="shared" ref="M17" si="6">L17*5</f>
-        <v>5</v>
+        <f t="shared" ref="M17" si="10">L17*5</f>
+        <v>15</v>
       </c>
       <c r="N17" s="51">
-        <v>10</v>
-      </c>
-      <c r="O17" s="73" t="s">
-        <v>122</v>
+        <v>100</v>
+      </c>
+      <c r="O17" s="63" t="s">
+        <v>69</v>
       </c>
       <c r="P17" s="52">
-        <v>0.1176</v>
+        <v>8.9999999999999998E-4</v>
       </c>
       <c r="Q17" s="52">
-        <f t="shared" ref="Q17" si="7">P17*N17</f>
-        <v>1.1759999999999999</v>
+        <f t="shared" ref="Q17" si="11">P17*N17</f>
+        <v>0.09</v>
       </c>
       <c r="R17" s="51"/>
       <c r="S17" s="59"/>
     </row>
-    <row r="18" spans="1:19" ht="24" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A18" s="1"/>
       <c r="B18" s="46">
         <f>ROW(B18) - ROW($B$9)</f>
         <v>9</v>
       </c>
       <c r="C18" s="53" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D18" s="37" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="E18" s="37" t="s">
-        <v>44</v>
-      </c>
-      <c r="F18" s="51" t="s">
-        <v>124</v>
+        <v>79</v>
+      </c>
+      <c r="F18" s="37" t="s">
+        <v>80</v>
       </c>
       <c r="G18" s="37" t="s">
-        <v>58</v>
+        <v>81</v>
       </c>
       <c r="H18" s="37" t="s">
+        <v>41</v>
+      </c>
+      <c r="I18" s="37" t="s">
+        <v>99</v>
+      </c>
+      <c r="J18" s="37" t="s">
+        <v>98</v>
+      </c>
+      <c r="K18" s="37" t="s">
         <v>82</v>
       </c>
-      <c r="I18" s="37" t="s">
-        <v>119</v>
-      </c>
-      <c r="J18" s="37" t="s">
-        <v>94</v>
-      </c>
-      <c r="K18" s="37"/>
       <c r="L18" s="37">
         <v>1</v>
       </c>
@@ -2174,484 +2112,261 @@
         <v>5</v>
       </c>
       <c r="N18" s="37">
-        <v>6</v>
-      </c>
-      <c r="O18" s="73" t="s">
-        <v>122</v>
+        <v>100</v>
+      </c>
+      <c r="O18" s="62" t="s">
+        <v>69</v>
       </c>
       <c r="P18" s="38">
-        <v>1.9235</v>
+        <v>8.9999999999999998E-4</v>
       </c>
       <c r="Q18" s="38">
         <f>P18*N18</f>
-        <v>11.541</v>
+        <v>0.09</v>
       </c>
       <c r="R18" s="37"/>
       <c r="S18" s="59"/>
     </row>
-    <row r="19" spans="1:19" ht="36" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A19" s="1"/>
       <c r="B19" s="47">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="B19" si="12">ROW(B19) - ROW($B$9)</f>
         <v>10</v>
       </c>
-      <c r="C19" s="54" t="s">
-        <v>15</v>
+      <c r="C19" s="53" t="s">
+        <v>13</v>
       </c>
       <c r="D19" s="51" t="s">
-        <v>28</v>
+        <v>83</v>
       </c>
       <c r="E19" s="51" t="s">
-        <v>45</v>
+        <v>84</v>
       </c>
       <c r="F19" s="51" t="s">
-        <v>59</v>
+        <v>33</v>
       </c>
       <c r="G19" s="51" t="s">
+        <v>85</v>
+      </c>
+      <c r="H19" s="51" t="s">
+        <v>86</v>
+      </c>
+      <c r="I19" s="51" t="s">
+        <v>66</v>
+      </c>
+      <c r="J19" s="51" t="s">
+        <v>87</v>
+      </c>
+      <c r="K19" s="51" t="s">
+        <v>88</v>
+      </c>
+      <c r="L19" s="51">
+        <v>4</v>
+      </c>
+      <c r="M19" s="51">
+        <f t="shared" ref="M19" si="13">L19*5</f>
+        <v>20</v>
+      </c>
+      <c r="N19" s="51">
+        <v>40</v>
+      </c>
+      <c r="O19" s="63" t="s">
         <v>69</v>
       </c>
-      <c r="H19" s="51" t="s">
-        <v>83</v>
-      </c>
-      <c r="I19" s="51" t="s">
-        <v>119</v>
-      </c>
-      <c r="J19" s="51" t="s">
-        <v>95</v>
-      </c>
-      <c r="K19" s="51"/>
-      <c r="L19" s="51">
-        <v>1</v>
-      </c>
-      <c r="M19" s="51">
-        <f t="shared" ref="M19" si="8">L19*5</f>
-        <v>5</v>
-      </c>
-      <c r="N19" s="51">
-        <v>20</v>
-      </c>
-      <c r="O19" s="73" t="s">
-        <v>122</v>
-      </c>
       <c r="P19" s="52">
-        <v>2.1499999999999998E-2</v>
+        <v>1.0999999999999999E-2</v>
       </c>
       <c r="Q19" s="52">
-        <f t="shared" ref="Q19" si="9">P19*N19</f>
-        <v>0.42999999999999994</v>
+        <f t="shared" ref="Q19" si="14">P19*N19</f>
+        <v>0.43999999999999995</v>
       </c>
       <c r="R19" s="51"/>
       <c r="S19" s="59"/>
     </row>
-    <row r="20" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:19" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1"/>
-      <c r="B20" s="46">
-        <f>ROW(B20) - ROW($B$9)</f>
+      <c r="B20" s="47">
+        <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="C20" s="53" t="s">
-        <v>16</v>
-      </c>
-      <c r="D20" s="37" t="s">
-        <v>29</v>
-      </c>
-      <c r="E20" s="37" t="s">
-        <v>46</v>
+      <c r="C20" s="54" t="s">
+        <v>65</v>
+      </c>
+      <c r="D20" s="51" t="s">
+        <v>20</v>
+      </c>
+      <c r="E20" s="51" t="s">
+        <v>27</v>
       </c>
       <c r="F20" s="37" t="s">
-        <v>60</v>
-      </c>
-      <c r="G20" s="37" t="s">
         <v>70</v>
       </c>
-      <c r="H20" s="37" t="s">
-        <v>76</v>
-      </c>
-      <c r="I20" s="37" t="s">
-        <v>119</v>
-      </c>
-      <c r="J20" s="37" t="s">
-        <v>96</v>
-      </c>
-      <c r="K20" s="37" t="s">
+      <c r="G20" s="51" t="s">
+        <v>39</v>
+      </c>
+      <c r="H20" s="51" t="s">
+        <v>45</v>
+      </c>
+      <c r="I20" s="51" t="s">
+        <v>66</v>
+      </c>
+      <c r="J20" s="51" t="s">
+        <v>51</v>
+      </c>
+      <c r="K20" s="51"/>
+      <c r="L20" s="51">
+        <v>3</v>
+      </c>
+      <c r="M20" s="51">
+        <f t="shared" ref="M20:M21" si="15">L20*5</f>
+        <v>15</v>
+      </c>
+      <c r="N20" s="51">
+        <v>20</v>
+      </c>
+      <c r="O20" s="62" t="s">
+        <v>69</v>
+      </c>
+      <c r="P20" s="52">
+        <v>5.5500000000000001E-2</v>
+      </c>
+      <c r="Q20" s="52">
+        <f t="shared" ref="Q20:Q21" si="16">P20*N20</f>
+        <v>1.1100000000000001</v>
+      </c>
+      <c r="R20" s="51"/>
+      <c r="S20" s="39"/>
+    </row>
+    <row r="21" spans="1:19" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="1"/>
+      <c r="B21" s="64">
+        <v>12</v>
+      </c>
+      <c r="C21" s="54" t="s">
+        <v>100</v>
+      </c>
+      <c r="D21" s="51" t="s">
+        <v>66</v>
+      </c>
+      <c r="E21" s="51" t="s">
+        <v>101</v>
+      </c>
+      <c r="F21" s="37" t="s">
+        <v>66</v>
+      </c>
+      <c r="G21" s="51" t="s">
+        <v>102</v>
+      </c>
+      <c r="H21" s="51" t="s">
+        <v>103</v>
+      </c>
+      <c r="I21" s="51" t="s">
+        <v>66</v>
+      </c>
+      <c r="J21" s="51" t="s">
         <v>104</v>
       </c>
-      <c r="L20" s="37">
-        <v>4</v>
-      </c>
-      <c r="M20" s="37">
-        <f>L20*5</f>
-        <v>20</v>
-      </c>
-      <c r="N20" s="37">
-        <v>40</v>
-      </c>
-      <c r="O20" s="73" t="s">
-        <v>122</v>
-      </c>
-      <c r="P20" s="38">
-        <v>2.1700000000000001E-2</v>
-      </c>
-      <c r="Q20" s="38">
-        <f>P20*N20</f>
-        <v>0.86799999999999999</v>
-      </c>
-      <c r="R20" s="37"/>
-      <c r="S20" s="59"/>
-    </row>
-    <row r="21" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A21" s="1"/>
-      <c r="B21" s="47">
-        <f t="shared" si="0"/>
-        <v>12</v>
-      </c>
-      <c r="C21" s="54" t="s">
-        <v>16</v>
-      </c>
-      <c r="D21" s="51" t="s">
-        <v>30</v>
-      </c>
-      <c r="E21" s="51" t="s">
-        <v>47</v>
-      </c>
-      <c r="F21" s="51" t="s">
-        <v>61</v>
-      </c>
-      <c r="G21" s="71" t="s">
-        <v>71</v>
-      </c>
-      <c r="H21" s="51" t="s">
-        <v>84</v>
-      </c>
-      <c r="I21" s="51" t="s">
-        <v>125</v>
-      </c>
-      <c r="J21" s="51" t="s">
-        <v>126</v>
-      </c>
       <c r="K21" s="51" t="s">
-        <v>105</v>
+        <v>66</v>
       </c>
       <c r="L21" s="51">
         <v>1</v>
       </c>
       <c r="M21" s="51">
-        <f t="shared" ref="M21" si="10">L21*5</f>
+        <f t="shared" si="15"/>
         <v>5</v>
       </c>
       <c r="N21" s="51">
-        <v>100</v>
-      </c>
-      <c r="O21" s="73" t="s">
-        <v>122</v>
+        <v>10</v>
+      </c>
+      <c r="O21" s="62" t="s">
+        <v>69</v>
       </c>
       <c r="P21" s="52">
-        <v>5.0000000000000001E-4</v>
+        <v>8.3199999999999996E-2</v>
       </c>
       <c r="Q21" s="52">
-        <f t="shared" ref="Q21" si="11">P21*N21</f>
-        <v>0.05</v>
+        <f t="shared" si="16"/>
+        <v>0.83199999999999996</v>
       </c>
       <c r="R21" s="51"/>
-      <c r="S21" s="59"/>
+      <c r="S21" s="39"/>
     </row>
-    <row r="22" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1"/>
-      <c r="B22" s="46">
-        <f>ROW(B22) - ROW($B$9)</f>
-        <v>13</v>
-      </c>
-      <c r="C22" s="54" t="s">
-        <v>16</v>
-      </c>
-      <c r="D22" s="37" t="s">
-        <v>31</v>
-      </c>
-      <c r="E22" s="37" t="s">
-        <v>48</v>
-      </c>
-      <c r="F22" s="37" t="s">
-        <v>61</v>
-      </c>
-      <c r="G22" s="37" t="s">
-        <v>72</v>
-      </c>
-      <c r="H22" s="37" t="s">
-        <v>76</v>
-      </c>
-      <c r="I22" s="37" t="s">
-        <v>119</v>
-      </c>
-      <c r="J22" s="37" t="s">
-        <v>97</v>
-      </c>
-      <c r="K22" s="37" t="s">
-        <v>106</v>
-      </c>
-      <c r="L22" s="37">
-        <v>1</v>
-      </c>
-      <c r="M22" s="37">
-        <f>L22*5</f>
+      <c r="B22" s="40"/>
+      <c r="C22" s="41"/>
+      <c r="D22" s="42"/>
+      <c r="E22" s="43"/>
+      <c r="F22" s="44"/>
+      <c r="G22" s="45"/>
+      <c r="H22" s="44"/>
+      <c r="I22" s="45"/>
+      <c r="J22" s="44"/>
+      <c r="K22" s="45"/>
+      <c r="L22" s="45"/>
+      <c r="M22" s="45"/>
+      <c r="N22" s="73" t="s">
         <v>5</v>
       </c>
-      <c r="N22" s="37">
-        <v>100</v>
-      </c>
-      <c r="O22" s="73" t="s">
-        <v>122</v>
-      </c>
-      <c r="P22" s="38">
-        <v>6.9999999999999999E-4</v>
-      </c>
-      <c r="Q22" s="38">
-        <f>P22*N22</f>
-        <v>6.9999999999999993E-2</v>
-      </c>
-      <c r="R22" s="37"/>
-      <c r="S22" s="59"/>
+      <c r="O22" s="74"/>
+      <c r="P22" s="74"/>
+      <c r="Q22" s="48">
+        <f>SUM(Q10:Q21)</f>
+        <v>9.0329999999999995</v>
+      </c>
+      <c r="R22" s="69"/>
+      <c r="S22" s="70"/>
     </row>
-    <row r="23" spans="1:19" ht="24" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1"/>
-      <c r="B23" s="47">
-        <f t="shared" si="0"/>
-        <v>14</v>
-      </c>
-      <c r="C23" s="54" t="s">
-        <v>16</v>
-      </c>
-      <c r="D23" s="51" t="s">
-        <v>32</v>
-      </c>
-      <c r="E23" s="51" t="s">
-        <v>49</v>
-      </c>
-      <c r="F23" s="51" t="s">
-        <v>61</v>
-      </c>
-      <c r="G23" s="51" t="s">
-        <v>73</v>
-      </c>
-      <c r="H23" s="51" t="s">
-        <v>85</v>
-      </c>
-      <c r="I23" s="51" t="s">
-        <v>119</v>
-      </c>
-      <c r="J23" s="51" t="s">
-        <v>98</v>
-      </c>
-      <c r="K23" s="51" t="s">
-        <v>107</v>
-      </c>
-      <c r="L23" s="51">
-        <v>1</v>
-      </c>
-      <c r="M23" s="51">
-        <f t="shared" ref="M23" si="12">L23*5</f>
-        <v>5</v>
-      </c>
-      <c r="N23" s="51">
-        <v>100</v>
-      </c>
-      <c r="O23" s="73" t="s">
-        <v>122</v>
-      </c>
-      <c r="P23" s="52">
-        <v>5.9999999999999995E-4</v>
-      </c>
-      <c r="Q23" s="52">
-        <f t="shared" ref="Q23" si="13">P23*N23</f>
-        <v>0.06</v>
-      </c>
-      <c r="R23" s="51"/>
-      <c r="S23" s="59"/>
-    </row>
-    <row r="24" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A24" s="1"/>
-      <c r="B24" s="46">
-        <f>ROW(B24) - ROW($B$9)</f>
-        <v>15</v>
-      </c>
-      <c r="C24" s="53" t="s">
-        <v>17</v>
-      </c>
-      <c r="D24" s="74" t="s">
-        <v>33</v>
-      </c>
-      <c r="E24" s="74" t="s">
-        <v>50</v>
-      </c>
-      <c r="F24" s="74" t="s">
-        <v>124</v>
-      </c>
-      <c r="G24" s="74" t="s">
-        <v>17</v>
-      </c>
-      <c r="H24" s="74" t="s">
-        <v>119</v>
-      </c>
-      <c r="I24" s="74" t="s">
-        <v>119</v>
-      </c>
-      <c r="J24" s="74" t="s">
-        <v>119</v>
-      </c>
-      <c r="K24" s="74"/>
-      <c r="L24" s="74">
-        <v>1</v>
-      </c>
-      <c r="M24" s="74">
-        <f>L24*5</f>
-        <v>5</v>
-      </c>
-      <c r="N24" s="74" t="s">
-        <v>119</v>
-      </c>
-      <c r="O24" s="74" t="s">
-        <v>119</v>
-      </c>
-      <c r="P24" s="75" t="s">
-        <v>119</v>
-      </c>
-      <c r="Q24" s="75" t="s">
-        <v>119</v>
-      </c>
-      <c r="R24" s="74"/>
-      <c r="S24" s="72"/>
-    </row>
-    <row r="25" spans="1:19" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="1"/>
-      <c r="B25" s="47">
-        <f t="shared" si="0"/>
-        <v>16</v>
-      </c>
-      <c r="C25" s="54" t="s">
-        <v>118</v>
-      </c>
-      <c r="D25" s="51" t="s">
-        <v>34</v>
-      </c>
-      <c r="E25" s="51" t="s">
-        <v>51</v>
-      </c>
-      <c r="F25" s="37" t="s">
-        <v>124</v>
-      </c>
-      <c r="G25" s="51" t="s">
-        <v>74</v>
-      </c>
-      <c r="H25" s="51" t="s">
-        <v>86</v>
-      </c>
-      <c r="I25" s="51" t="s">
-        <v>119</v>
-      </c>
-      <c r="J25" s="51" t="s">
-        <v>99</v>
-      </c>
-      <c r="K25" s="51"/>
-      <c r="L25" s="51">
-        <v>3</v>
-      </c>
-      <c r="M25" s="51">
-        <f t="shared" ref="M25" si="14">L25*5</f>
-        <v>15</v>
-      </c>
-      <c r="N25" s="51">
-        <v>20</v>
-      </c>
-      <c r="O25" s="73" t="s">
-        <v>122</v>
-      </c>
-      <c r="P25" s="52">
-        <v>5.5500000000000001E-2</v>
-      </c>
-      <c r="Q25" s="52">
-        <f t="shared" ref="Q25" si="15">P25*N25</f>
-        <v>1.1100000000000001</v>
-      </c>
-      <c r="R25" s="51"/>
-      <c r="S25" s="39"/>
-    </row>
-    <row r="26" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="1"/>
-      <c r="B26" s="40"/>
-      <c r="C26" s="41"/>
-      <c r="D26" s="42"/>
-      <c r="E26" s="43"/>
-      <c r="F26" s="44"/>
-      <c r="G26" s="45"/>
-      <c r="H26" s="44"/>
-      <c r="I26" s="45"/>
-      <c r="J26" s="44"/>
-      <c r="K26" s="45"/>
-      <c r="L26" s="45"/>
-      <c r="M26" s="45"/>
-      <c r="N26" s="68" t="s">
-        <v>5</v>
-      </c>
-      <c r="O26" s="69"/>
-      <c r="P26" s="69"/>
-      <c r="Q26" s="48">
-        <f>SUM(Q10:Q25)</f>
-        <v>22.001499999999997</v>
-      </c>
-      <c r="R26" s="64"/>
-      <c r="S26" s="65"/>
-    </row>
-    <row r="27" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="1"/>
-      <c r="B27" s="25"/>
-      <c r="C27" s="36"/>
-      <c r="D27" s="9"/>
-      <c r="E27" s="10"/>
-      <c r="F27" s="10"/>
-      <c r="G27" s="10"/>
-      <c r="H27" s="10"/>
-      <c r="I27" s="10"/>
-      <c r="J27" s="10"/>
-      <c r="K27" s="10"/>
-      <c r="L27" s="10"/>
-      <c r="M27" s="10"/>
-      <c r="N27" s="68" t="s">
+      <c r="B23" s="25"/>
+      <c r="C23" s="36"/>
+      <c r="D23" s="9"/>
+      <c r="E23" s="10"/>
+      <c r="F23" s="10"/>
+      <c r="G23" s="10"/>
+      <c r="H23" s="10"/>
+      <c r="I23" s="10"/>
+      <c r="J23" s="10"/>
+      <c r="K23" s="10"/>
+      <c r="L23" s="10"/>
+      <c r="M23" s="10"/>
+      <c r="N23" s="73" t="s">
         <v>6</v>
       </c>
-      <c r="O27" s="69"/>
-      <c r="P27" s="69"/>
-      <c r="Q27" s="49">
-        <f>Q26/5</f>
-        <v>4.4002999999999997</v>
-      </c>
-      <c r="R27" s="66"/>
-      <c r="S27" s="67"/>
+      <c r="O23" s="74"/>
+      <c r="P23" s="74"/>
+      <c r="Q23" s="49">
+        <f>Q22/5</f>
+        <v>1.8066</v>
+      </c>
+      <c r="R23" s="71"/>
+      <c r="S23" s="72"/>
     </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="K1:S1"/>
     <mergeCell ref="S3:S8"/>
-    <mergeCell ref="R26:S27"/>
-    <mergeCell ref="N26:P26"/>
-    <mergeCell ref="N27:P27"/>
+    <mergeCell ref="R22:S23"/>
+    <mergeCell ref="N22:P22"/>
+    <mergeCell ref="N23:P23"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="O10" r:id="rId1"/>
-    <hyperlink ref="O11" r:id="rId2"/>
-    <hyperlink ref="O12" r:id="rId3"/>
-    <hyperlink ref="O13" r:id="rId4"/>
-    <hyperlink ref="O14" r:id="rId5"/>
+    <hyperlink ref="O11" r:id="rId1"/>
+    <hyperlink ref="O10" r:id="rId2"/>
+    <hyperlink ref="O14" r:id="rId3"/>
+    <hyperlink ref="O15" r:id="rId4"/>
+    <hyperlink ref="O20" r:id="rId5"/>
     <hyperlink ref="O16" r:id="rId6"/>
-    <hyperlink ref="O17" r:id="rId7"/>
-    <hyperlink ref="O18" r:id="rId8"/>
-    <hyperlink ref="O19" r:id="rId9"/>
-    <hyperlink ref="O20" r:id="rId10"/>
+    <hyperlink ref="O18" r:id="rId7"/>
+    <hyperlink ref="O19" r:id="rId8"/>
+    <hyperlink ref="O13" r:id="rId9"/>
+    <hyperlink ref="O17" r:id="rId10"/>
     <hyperlink ref="O21" r:id="rId11"/>
-    <hyperlink ref="O22" r:id="rId12"/>
-    <hyperlink ref="O23" r:id="rId13"/>
-    <hyperlink ref="O25" r:id="rId14"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId15"/>
-  <drawing r:id="rId16"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId12"/>
+  <drawing r:id="rId13"/>
 </worksheet>
 </file>
</xml_diff>